<commit_message>
Group B: 6901 / 6805 / 6806 / 6809 SPECs (existing NWO / NPSM / NPTF / JIC swivel legs) + Brennan-record cells: 48 configurations, checks clean
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Sbz7LkX6Jr9QuSxTU76dzT
</commit_message>
<xml_diff>
--- a/tools/_out/groupB_20261021/stage/04_DESIGN_TABLES/DesignTable_6805.xlsx
+++ b/tools/_out/groupB_20261021/stage/04_DESIGN_TABLES/DesignTable_6805.xlsx
@@ -1008,7 +1008,7 @@
         <v>1.47</v>
       </c>
       <c r="C9" s="4" t="n">
-        <v>0.63</v>
+        <v>1.02</v>
       </c>
       <c r="D9" s="4" t="n">
         <v>0.88</v>
@@ -1054,12 +1054,12 @@
       </c>
       <c r="P9" s="4" t="inlineStr">
         <is>
-          <t>Air-Way s138 only (double-pass 18 rows); ORB end: measured/published groove set + MS51527 J2; female NPTF per ANSI B1.20.3</t>
+          <t>[BRENNAN-CELL 2026-10-21: N1@DRIVE] Air-Way s138 only (double-pass 18 rows); ORB end: measured/published groove set + MS51527 J2; female NPTF per ANSI B1.20.3</t>
         </is>
       </c>
       <c r="Q9" s="4" t="inlineStr">
         <is>
-          <t>N1 printed 0.63 both passes (non-FG prints 1.02; a 3/8-18 female leg ~1.02) - as-printed, likely typo</t>
+          <t>N1 printed 0.63 both passes (non-FG prints 1.02; a 3/8-18 female leg ~1.02) - as-printed, likely typo | Air-Way N1 0.63 cannot be built (female -06 port MS51503 P1 0.68 is longer than the leg) -&gt; Brennan CAD record N 1.02 (= Air-Way's own non-FG 6805-08-06-NWO row; user Q1 2026-10-20 "use brennans")</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
@@ -1070,6 +1070,11 @@
       <c r="S9" t="inlineStr">
         <is>
           <t>6805-08-06-NWO-FG</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>BRENNAN</t>
         </is>
       </c>
     </row>
@@ -1848,9 +1853,18 @@
           <t>6805-04-02-NWO-FG</t>
         </is>
       </c>
+      <c r="B21" t="n">
+        <v>1.19</v>
+      </c>
+      <c r="C21" t="n">
+        <v>0.66</v>
+      </c>
       <c r="D21" t="n">
         <v>0.5629999999999999</v>
       </c>
+      <c r="E21" t="n">
+        <v>0.5620000000000001</v>
+      </c>
       <c r="F21" t="n">
         <v>0.172</v>
       </c>
@@ -1878,12 +1892,12 @@
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>[A1/A9 TAPDRILL 2026-10-21: TAPDRILL@BORE] [BRENNAN-CAD 2026-10-21: C4HEX@HEX, D@BORE, ORB_GRVDIA@DRIVE, THDMAJ_A@DRIVE, THDMAJ_B@DRIVE] OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); Air-Way has this size only as 6805-04-02-NWO (differs by -FG/-UNPL suffix) -&gt; dims NOT copied</t>
+          <t>[BRENNAN-CAD 2026-10-21 group B: M17@DRIVE, N1@DRIVE, Y1@REF] [A1/A9 TAPDRILL 2026-10-21: TAPDRILL@BORE] [BRENNAN-CAD 2026-10-21: C4HEX@HEX, D@BORE, ORB_GRVDIA@DRIVE, THDMAJ_A@DRIVE, THDMAJ_B@DRIVE] OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); Air-Way has this size only as 6805-04-02-NWO (differs by -FG/-UNPL suffix) -&gt; dims NOT copied</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>BUILD-NEAR: forged (-FG) and non-FG variants differ in length on other series, so 6805-04-02-NWO dims are NOT assumed; confirm before modelling | Brennan CAD record 6805-04-02-NWO-FG (PARTcommunity / CADENAS, C4HEX@HEX=C, D@BORE=BD, ORB_GRVDIA@DRIVE=HL, THDMAJ_A@DRIVE=ATHD, THDMAJ_B@DRIVE=BTHD; user 2026-10-21 "yes you can use them following my rule") | TAPDRILL@BORE = Air-Way per-size tap drill -02 0.33 (A1)</t>
+          <t>BUILD-NEAR: forged (-FG) and non-FG variants differ in length on other series, so 6805-04-02-NWO dims are NOT assumed; confirm before modelling | Brennan CAD record 6805-04-02-NWO-FG (PARTcommunity / CADENAS, C4HEX@HEX=C, D@BORE=BD, ORB_GRVDIA@DRIVE=HL, THDMAJ_A@DRIVE=ATHD, THDMAJ_B@DRIVE=BTHD; user 2026-10-21 "yes you can use them following my rule") | TAPDRILL@BORE = Air-Way per-size tap drill -02 0.33 (A1) | Brennan CAD record 6805-04-02-NWO-FG (PARTcommunity / CADENAS, group B 2026-10-21: M17@DRIVE=M7, N1@DRIVE=N, Y1@REF=Y; user 2026-10-21 "yes you can use them following my rule")</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
@@ -1908,9 +1922,18 @@
           <t>6805-04-04-NWO-FG</t>
         </is>
       </c>
+      <c r="B22" t="n">
+        <v>1.26</v>
+      </c>
+      <c r="C22" t="n">
+        <v>0.88</v>
+      </c>
       <c r="D22" t="n">
         <v>0.5629999999999999</v>
       </c>
+      <c r="E22" t="n">
+        <v>0.75</v>
+      </c>
       <c r="F22" t="n">
         <v>0.172</v>
       </c>
@@ -1938,12 +1961,12 @@
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>[A1/A9 TAPDRILL 2026-10-21: TAPDRILL@BORE] [BRENNAN-CAD 2026-10-21: C4HEX@HEX, D@BORE, ORB_GRVDIA@DRIVE, THDMAJ_A@DRIVE, THDMAJ_B@DRIVE] OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); Air-Way has this size only as 6805-04-04-NWO (differs by -FG/-UNPL suffix) -&gt; dims NOT copied</t>
+          <t>[BRENNAN-CAD 2026-10-21 group B: M17@DRIVE, N1@DRIVE, Y1@REF] [A1/A9 TAPDRILL 2026-10-21: TAPDRILL@BORE] [BRENNAN-CAD 2026-10-21: C4HEX@HEX, D@BORE, ORB_GRVDIA@DRIVE, THDMAJ_A@DRIVE, THDMAJ_B@DRIVE] OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); Air-Way has this size only as 6805-04-04-NWO (differs by -FG/-UNPL suffix) -&gt; dims NOT copied</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>BUILD-NEAR: forged (-FG) and non-FG variants differ in length on other series, so 6805-04-04-NWO dims are NOT assumed; confirm before modelling | Brennan CAD record 6805-04-04-NWO-FG (PARTcommunity / CADENAS, C4HEX@HEX=C, D@BORE=BD, ORB_GRVDIA@DRIVE=HL, THDMAJ_A@DRIVE=ATHD, THDMAJ_B@DRIVE=BTHD; user 2026-10-21 "yes you can use them following my rule") | TAPDRILL@BORE = Air-Way per-size tap drill -04 0.43 (A1)</t>
+          <t>BUILD-NEAR: forged (-FG) and non-FG variants differ in length on other series, so 6805-04-04-NWO dims are NOT assumed; confirm before modelling | Brennan CAD record 6805-04-04-NWO-FG (PARTcommunity / CADENAS, C4HEX@HEX=C, D@BORE=BD, ORB_GRVDIA@DRIVE=HL, THDMAJ_A@DRIVE=ATHD, THDMAJ_B@DRIVE=BTHD; user 2026-10-21 "yes you can use them following my rule") | TAPDRILL@BORE = Air-Way per-size tap drill -04 0.43 (A1) | Brennan CAD record 6805-04-04-NWO-FG (PARTcommunity / CADENAS, group B 2026-10-21: M17@DRIVE=M7, N1@DRIVE=N, Y1@REF=Y; user 2026-10-21 "yes you can use them following my rule")</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
@@ -1968,9 +1991,18 @@
           <t>6805-06-06-NWO-FG</t>
         </is>
       </c>
+      <c r="B23" t="n">
+        <v>1.41</v>
+      </c>
+      <c r="C23" t="n">
+        <v>1.02</v>
+      </c>
       <c r="D23" t="n">
         <v>0.6879999999999999</v>
       </c>
+      <c r="E23" t="n">
+        <v>0.875</v>
+      </c>
       <c r="F23" t="n">
         <v>0.297</v>
       </c>
@@ -1998,12 +2030,12 @@
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>[A1/A9 TAPDRILL 2026-10-21: TAPDRILL@BORE] [BRENNAN-CAD 2026-10-21: C4HEX@HEX, D@BORE, ORB_GRVDIA@DRIVE, THDMAJ_A@DRIVE, THDMAJ_B@DRIVE] OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); Air-Way has this size only as 6805-06-06-NWO (differs by -FG/-UNPL suffix) -&gt; dims NOT copied</t>
+          <t>[BRENNAN-CAD 2026-10-21 group B: M17@DRIVE, N1@DRIVE, Y1@REF] [A1/A9 TAPDRILL 2026-10-21: TAPDRILL@BORE] [BRENNAN-CAD 2026-10-21: C4HEX@HEX, D@BORE, ORB_GRVDIA@DRIVE, THDMAJ_A@DRIVE, THDMAJ_B@DRIVE] OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); Air-Way has this size only as 6805-06-06-NWO (differs by -FG/-UNPL suffix) -&gt; dims NOT copied</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>BUILD-NEAR: forged (-FG) and non-FG variants differ in length on other series, so 6805-06-06-NWO dims are NOT assumed; confirm before modelling | Brennan CAD record 6805-06-06-NWO-FG (PARTcommunity / CADENAS, C4HEX@HEX=C, D@BORE=BD, ORB_GRVDIA@DRIVE=HL, THDMAJ_A@DRIVE=ATHD, THDMAJ_B@DRIVE=BTHD; user 2026-10-21 "yes you can use them following my rule") | TAPDRILL@BORE = Air-Way per-size tap drill -06 0.57 (A1)</t>
+          <t>BUILD-NEAR: forged (-FG) and non-FG variants differ in length on other series, so 6805-06-06-NWO dims are NOT assumed; confirm before modelling | Brennan CAD record 6805-06-06-NWO-FG (PARTcommunity / CADENAS, C4HEX@HEX=C, D@BORE=BD, ORB_GRVDIA@DRIVE=HL, THDMAJ_A@DRIVE=ATHD, THDMAJ_B@DRIVE=BTHD; user 2026-10-21 "yes you can use them following my rule") | TAPDRILL@BORE = Air-Way per-size tap drill -06 0.57 (A1) | Brennan CAD record 6805-06-06-NWO-FG (PARTcommunity / CADENAS, group B 2026-10-21: M17@DRIVE=M7, N1@DRIVE=N, Y1@REF=Y; user 2026-10-21 "yes you can use them following my rule")</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
@@ -2028,9 +2060,18 @@
           <t>6805-08-08-NWO-FG</t>
         </is>
       </c>
+      <c r="B24" t="n">
+        <v>1.62</v>
+      </c>
+      <c r="C24" t="n">
+        <v>1.23</v>
+      </c>
       <c r="D24" t="n">
         <v>0.875</v>
       </c>
+      <c r="E24" t="n">
+        <v>1.062</v>
+      </c>
       <c r="F24" t="n">
         <v>0.391</v>
       </c>
@@ -2058,12 +2099,12 @@
       </c>
       <c r="P24" t="inlineStr">
         <is>
-          <t>[A1/A9 TAPDRILL 2026-10-21: TAPDRILL@BORE] [BRENNAN-CAD 2026-10-21: C4HEX@HEX, D@BORE, ORB_GRVDIA@DRIVE, THDMAJ_A@DRIVE, THDMAJ_B@DRIVE] OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); Air-Way has this size only as 6805-08-08-NWO (differs by -FG/-UNPL suffix) -&gt; dims NOT copied</t>
+          <t>[BRENNAN-CAD 2026-10-21 group B: M17@DRIVE, N1@DRIVE, Y1@REF] [A1/A9 TAPDRILL 2026-10-21: TAPDRILL@BORE] [BRENNAN-CAD 2026-10-21: C4HEX@HEX, D@BORE, ORB_GRVDIA@DRIVE, THDMAJ_A@DRIVE, THDMAJ_B@DRIVE] OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); Air-Way has this size only as 6805-08-08-NWO (differs by -FG/-UNPL suffix) -&gt; dims NOT copied</t>
         </is>
       </c>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>BUILD-NEAR: forged (-FG) and non-FG variants differ in length on other series, so 6805-08-08-NWO dims are NOT assumed; confirm before modelling | Brennan CAD record 6805-08-08-NWO-FG (PARTcommunity / CADENAS, C4HEX@HEX=C, D@BORE=BD, ORB_GRVDIA@DRIVE=HL, THDMAJ_A@DRIVE=ATHD, THDMAJ_B@DRIVE=BTHD; user 2026-10-21 "yes you can use them following my rule") | TAPDRILL@BORE = Air-Way per-size tap drill -08 0.7 (A1)</t>
+          <t>BUILD-NEAR: forged (-FG) and non-FG variants differ in length on other series, so 6805-08-08-NWO dims are NOT assumed; confirm before modelling | Brennan CAD record 6805-08-08-NWO-FG (PARTcommunity / CADENAS, C4HEX@HEX=C, D@BORE=BD, ORB_GRVDIA@DRIVE=HL, THDMAJ_A@DRIVE=ATHD, THDMAJ_B@DRIVE=BTHD; user 2026-10-21 "yes you can use them following my rule") | TAPDRILL@BORE = Air-Way per-size tap drill -08 0.7 (A1) | Brennan CAD record 6805-08-08-NWO-FG (PARTcommunity / CADENAS, group B 2026-10-21: M17@DRIVE=M7, N1@DRIVE=N, Y1@REF=Y; user 2026-10-21 "yes you can use them following my rule")</t>
         </is>
       </c>
       <c r="R24" t="inlineStr">
@@ -2088,9 +2129,18 @@
           <t>6805-10-08-NWO-FG</t>
         </is>
       </c>
+      <c r="B25" t="n">
+        <v>1.78</v>
+      </c>
+      <c r="C25" t="n">
+        <v>1.23</v>
+      </c>
       <c r="D25" t="n">
         <v>1</v>
       </c>
+      <c r="E25" t="n">
+        <v>1.062</v>
+      </c>
       <c r="F25" t="n">
         <v>0.484</v>
       </c>
@@ -2118,12 +2168,12 @@
       </c>
       <c r="P25" t="inlineStr">
         <is>
-          <t>[A1/A9 TAPDRILL 2026-10-21: TAPDRILL@BORE] [BRENNAN-CAD 2026-10-21: C4HEX@HEX, D@BORE, ORB_GRVDIA@DRIVE, THDMAJ_A@DRIVE, THDMAJ_B@DRIVE] OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); Air-Way has this size only as 6805-10-08-NWO (differs by -FG/-UNPL suffix) -&gt; dims NOT copied</t>
+          <t>[BRENNAN-CAD 2026-10-21 group B: M17@DRIVE, N1@DRIVE, Y1@REF] [A1/A9 TAPDRILL 2026-10-21: TAPDRILL@BORE] [BRENNAN-CAD 2026-10-21: C4HEX@HEX, D@BORE, ORB_GRVDIA@DRIVE, THDMAJ_A@DRIVE, THDMAJ_B@DRIVE] OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); Air-Way has this size only as 6805-10-08-NWO (differs by -FG/-UNPL suffix) -&gt; dims NOT copied</t>
         </is>
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>BUILD-NEAR: forged (-FG) and non-FG variants differ in length on other series, so 6805-10-08-NWO dims are NOT assumed; confirm before modelling | Brennan CAD record 6805-10-08-NWO-FG (PARTcommunity / CADENAS, C4HEX@HEX=C, D@BORE=BD, ORB_GRVDIA@DRIVE=HL, THDMAJ_A@DRIVE=ATHD, THDMAJ_B@DRIVE=BTHD; user 2026-10-21 "yes you can use them following my rule") | TAPDRILL@BORE = Air-Way per-size tap drill -08 0.7 (A1)</t>
+          <t>BUILD-NEAR: forged (-FG) and non-FG variants differ in length on other series, so 6805-10-08-NWO dims are NOT assumed; confirm before modelling | Brennan CAD record 6805-10-08-NWO-FG (PARTcommunity / CADENAS, C4HEX@HEX=C, D@BORE=BD, ORB_GRVDIA@DRIVE=HL, THDMAJ_A@DRIVE=ATHD, THDMAJ_B@DRIVE=BTHD; user 2026-10-21 "yes you can use them following my rule") | TAPDRILL@BORE = Air-Way per-size tap drill -08 0.7 (A1) | Brennan CAD record 6805-10-08-NWO-FG (PARTcommunity / CADENAS, group B 2026-10-21: M17@DRIVE=M7, N1@DRIVE=N, Y1@REF=Y; user 2026-10-21 "yes you can use them following my rule")</t>
         </is>
       </c>
       <c r="R25" t="inlineStr">
@@ -2148,9 +2198,18 @@
           <t>6805-12-08-NWO-FG</t>
         </is>
       </c>
+      <c r="B26" t="n">
+        <v>1.94</v>
+      </c>
+      <c r="C26" t="n">
+        <v>1.23</v>
+      </c>
       <c r="D26" t="n">
         <v>1.25</v>
       </c>
+      <c r="E26" t="n">
+        <v>1.062</v>
+      </c>
       <c r="F26" t="n">
         <v>0.609</v>
       </c>
@@ -2178,12 +2237,12 @@
       </c>
       <c r="P26" t="inlineStr">
         <is>
-          <t>[A1/A9 TAPDRILL 2026-10-21: TAPDRILL@BORE] [BRENNAN-CAD 2026-10-21: C4HEX@HEX, D@BORE, ORB_GRVDIA@DRIVE, THDMAJ_A@DRIVE, THDMAJ_B@DRIVE] OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); Air-Way has this size only as 6805-12-08-NWO (differs by -FG/-UNPL suffix) -&gt; dims NOT copied</t>
+          <t>[BRENNAN-CAD 2026-10-21 group B: M17@DRIVE, N1@DRIVE, Y1@REF] [A1/A9 TAPDRILL 2026-10-21: TAPDRILL@BORE] [BRENNAN-CAD 2026-10-21: C4HEX@HEX, D@BORE, ORB_GRVDIA@DRIVE, THDMAJ_A@DRIVE, THDMAJ_B@DRIVE] OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); Air-Way has this size only as 6805-12-08-NWO (differs by -FG/-UNPL suffix) -&gt; dims NOT copied</t>
         </is>
       </c>
       <c r="Q26" t="inlineStr">
         <is>
-          <t>BUILD-NEAR: forged (-FG) and non-FG variants differ in length on other series, so 6805-12-08-NWO dims are NOT assumed; confirm before modelling | Brennan CAD record 6805-12-08-NWO-FG (PARTcommunity / CADENAS, C4HEX@HEX=C, D@BORE=BD, ORB_GRVDIA@DRIVE=HL, THDMAJ_A@DRIVE=ATHD, THDMAJ_B@DRIVE=BTHD; user 2026-10-21 "yes you can use them following my rule") | TAPDRILL@BORE = Air-Way per-size tap drill -08 0.7 (A1)</t>
+          <t>BUILD-NEAR: forged (-FG) and non-FG variants differ in length on other series, so 6805-12-08-NWO dims are NOT assumed; confirm before modelling | Brennan CAD record 6805-12-08-NWO-FG (PARTcommunity / CADENAS, C4HEX@HEX=C, D@BORE=BD, ORB_GRVDIA@DRIVE=HL, THDMAJ_A@DRIVE=ATHD, THDMAJ_B@DRIVE=BTHD; user 2026-10-21 "yes you can use them following my rule") | TAPDRILL@BORE = Air-Way per-size tap drill -08 0.7 (A1) | Brennan CAD record 6805-12-08-NWO-FG (PARTcommunity / CADENAS, group B 2026-10-21: M17@DRIVE=M7, N1@DRIVE=N, Y1@REF=Y; user 2026-10-21 "yes you can use them following my rule")</t>
         </is>
       </c>
       <c r="R26" t="inlineStr">
@@ -2208,9 +2267,18 @@
           <t>6805-16-12-NWO-FG</t>
         </is>
       </c>
+      <c r="B27" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="C27" t="n">
+        <v>1.36</v>
+      </c>
       <c r="D27" t="n">
         <v>1.5</v>
       </c>
+      <c r="E27" t="n">
+        <v>1.312</v>
+      </c>
       <c r="F27" t="n">
         <v>0.844</v>
       </c>
@@ -2238,12 +2306,12 @@
       </c>
       <c r="P27" t="inlineStr">
         <is>
-          <t>[A1/A9 TAPDRILL 2026-10-21: TAPDRILL@BORE] [BRENNAN-CAD 2026-10-21: C4HEX@HEX, D@BORE, ORB_GRVDIA@DRIVE, THDMAJ_A@DRIVE, THDMAJ_B@DRIVE] OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); Air-Way has this size only as 6805-16-12-NWO (differs by -FG/-UNPL suffix) -&gt; dims NOT copied</t>
+          <t>[BRENNAN-CAD 2026-10-21 group B: M17@DRIVE, N1@DRIVE, Y1@REF] [A1/A9 TAPDRILL 2026-10-21: TAPDRILL@BORE] [BRENNAN-CAD 2026-10-21: C4HEX@HEX, D@BORE, ORB_GRVDIA@DRIVE, THDMAJ_A@DRIVE, THDMAJ_B@DRIVE] OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); Air-Way has this size only as 6805-16-12-NWO (differs by -FG/-UNPL suffix) -&gt; dims NOT copied</t>
         </is>
       </c>
       <c r="Q27" t="inlineStr">
         <is>
-          <t>BUILD-NEAR: forged (-FG) and non-FG variants differ in length on other series, so 6805-16-12-NWO dims are NOT assumed; confirm before modelling | Brennan CAD record 6805-16-12-NWO-FG (PARTcommunity / CADENAS, C4HEX@HEX=C, D@BORE=BD, ORB_GRVDIA@DRIVE=HL, THDMAJ_A@DRIVE=ATHD, THDMAJ_B@DRIVE=BTHD; user 2026-10-21 "yes you can use them following my rule") | TAPDRILL@BORE = Air-Way per-size tap drill -12 0.91 (A1)</t>
+          <t>BUILD-NEAR: forged (-FG) and non-FG variants differ in length on other series, so 6805-16-12-NWO dims are NOT assumed; confirm before modelling | Brennan CAD record 6805-16-12-NWO-FG (PARTcommunity / CADENAS, C4HEX@HEX=C, D@BORE=BD, ORB_GRVDIA@DRIVE=HL, THDMAJ_A@DRIVE=ATHD, THDMAJ_B@DRIVE=BTHD; user 2026-10-21 "yes you can use them following my rule") | TAPDRILL@BORE = Air-Way per-size tap drill -12 0.91 (A1) | Brennan CAD record 6805-16-12-NWO-FG (PARTcommunity / CADENAS, group B 2026-10-21: M17@DRIVE=M7, N1@DRIVE=N, Y1@REF=Y; user 2026-10-21 "yes you can use them following my rule")</t>
         </is>
       </c>
       <c r="R27" t="inlineStr">
@@ -2268,9 +2336,18 @@
           <t>6805-16-16-NWO-FG</t>
         </is>
       </c>
+      <c r="B28" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="C28" t="n">
+        <v>1.62</v>
+      </c>
       <c r="D28" t="n">
         <v>1.5</v>
       </c>
+      <c r="E28" t="n">
+        <v>1.625</v>
+      </c>
       <c r="F28" t="n">
         <v>0.844</v>
       </c>
@@ -2298,12 +2375,12 @@
       </c>
       <c r="P28" t="inlineStr">
         <is>
-          <t>[A1/A9 TAPDRILL 2026-10-21: TAPDRILL@BORE] [BRENNAN-CAD 2026-10-21: C4HEX@HEX, D@BORE, ORB_GRVDIA@DRIVE, THDMAJ_A@DRIVE, THDMAJ_B@DRIVE] OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); Air-Way has this size only as 6805-16-16-NWO (differs by -FG/-UNPL suffix) -&gt; dims NOT copied</t>
+          <t>[BRENNAN-CAD 2026-10-21 group B: M17@DRIVE, N1@DRIVE, Y1@REF] [A1/A9 TAPDRILL 2026-10-21: TAPDRILL@BORE] [BRENNAN-CAD 2026-10-21: C4HEX@HEX, D@BORE, ORB_GRVDIA@DRIVE, THDMAJ_A@DRIVE, THDMAJ_B@DRIVE] OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); Air-Way has this size only as 6805-16-16-NWO (differs by -FG/-UNPL suffix) -&gt; dims NOT copied</t>
         </is>
       </c>
       <c r="Q28" t="inlineStr">
         <is>
-          <t>BUILD-NEAR: forged (-FG) and non-FG variants differ in length on other series, so 6805-16-16-NWO dims are NOT assumed; confirm before modelling | Brennan CAD record 6805-16-16-NWO-FG (PARTcommunity / CADENAS, C4HEX@HEX=C, D@BORE=BD, ORB_GRVDIA@DRIVE=HL, THDMAJ_A@DRIVE=ATHD, THDMAJ_B@DRIVE=BTHD; user 2026-10-21 "yes you can use them following my rule") | TAPDRILL@BORE = Air-Way per-size tap drill -16 1.14 (A1)</t>
+          <t>BUILD-NEAR: forged (-FG) and non-FG variants differ in length on other series, so 6805-16-16-NWO dims are NOT assumed; confirm before modelling | Brennan CAD record 6805-16-16-NWO-FG (PARTcommunity / CADENAS, C4HEX@HEX=C, D@BORE=BD, ORB_GRVDIA@DRIVE=HL, THDMAJ_A@DRIVE=ATHD, THDMAJ_B@DRIVE=BTHD; user 2026-10-21 "yes you can use them following my rule") | TAPDRILL@BORE = Air-Way per-size tap drill -16 1.14 (A1) | Brennan CAD record 6805-16-16-NWO-FG (PARTcommunity / CADENAS, group B 2026-10-21: M17@DRIVE=M7, N1@DRIVE=N, Y1@REF=Y; user 2026-10-21 "yes you can use them following my rule")</t>
         </is>
       </c>
       <c r="R28" t="inlineStr">
@@ -2328,9 +2405,18 @@
           <t>6805-20-20-NWO-FG</t>
         </is>
       </c>
+      <c r="B29" t="n">
+        <v>2.39</v>
+      </c>
+      <c r="C29" t="n">
+        <v>1.7</v>
+      </c>
       <c r="D29" t="n">
         <v>1.875</v>
       </c>
+      <c r="E29" t="n">
+        <v>1.875</v>
+      </c>
       <c r="F29" t="n">
         <v>1.078</v>
       </c>
@@ -2358,12 +2444,12 @@
       </c>
       <c r="P29" t="inlineStr">
         <is>
-          <t>[A1/A9 TAPDRILL 2026-10-21: TAPDRILL@BORE] [BRENNAN-CAD 2026-10-21: C4HEX@HEX, D@BORE, ORB_GRVDIA@DRIVE, THDMAJ_A@DRIVE, THDMAJ_B@DRIVE] OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); Air-Way has this size only as 6805-20-20-NWO (differs by -FG/-UNPL suffix) -&gt; dims NOT copied</t>
+          <t>[BRENNAN-CAD 2026-10-21 group B: M17@DRIVE, N1@DRIVE, Y1@REF] [A1/A9 TAPDRILL 2026-10-21: TAPDRILL@BORE] [BRENNAN-CAD 2026-10-21: C4HEX@HEX, D@BORE, ORB_GRVDIA@DRIVE, THDMAJ_A@DRIVE, THDMAJ_B@DRIVE] OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); Air-Way has this size only as 6805-20-20-NWO (differs by -FG/-UNPL suffix) -&gt; dims NOT copied</t>
         </is>
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>BUILD-NEAR: forged (-FG) and non-FG variants differ in length on other series, so 6805-20-20-NWO dims are NOT assumed; confirm before modelling | Brennan CAD record 6805-20-20-NWO-FG (PARTcommunity / CADENAS, C4HEX@HEX=C, D@BORE=BD, ORB_GRVDIA@DRIVE=HL, THDMAJ_A@DRIVE=ATHD, THDMAJ_B@DRIVE=BTHD; user 2026-10-21 "yes you can use them following my rule") | TAPDRILL@BORE = Air-Way per-size tap drill -20 1.48 (A1)</t>
+          <t>BUILD-NEAR: forged (-FG) and non-FG variants differ in length on other series, so 6805-20-20-NWO dims are NOT assumed; confirm before modelling | Brennan CAD record 6805-20-20-NWO-FG (PARTcommunity / CADENAS, C4HEX@HEX=C, D@BORE=BD, ORB_GRVDIA@DRIVE=HL, THDMAJ_A@DRIVE=ATHD, THDMAJ_B@DRIVE=BTHD; user 2026-10-21 "yes you can use them following my rule") | TAPDRILL@BORE = Air-Way per-size tap drill -20 1.48 (A1) | Brennan CAD record 6805-20-20-NWO-FG (PARTcommunity / CADENAS, group B 2026-10-21: M17@DRIVE=M7, N1@DRIVE=N, Y1@REF=Y; user 2026-10-21 "yes you can use them following my rule")</t>
         </is>
       </c>
       <c r="R29" t="inlineStr">

</xml_diff>